<commit_message>
Remove duplicate catalog models and correct video placement
</commit_message>
<xml_diff>
--- a/docs/MCCS_CF_Product_Specifications.xlsx
+++ b/docs/MCCS_CF_Product_Specifications.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF 产品规格" sheetId="1" r:id="Rdbfea55286d3440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购说明" sheetId="2" r:id="R39c5f267c19b41a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF 产品规格" sheetId="1" r:id="R38dba418bc9b43c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购说明" sheetId="2" r:id="R64c1203b4fd2442a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -271,8 +271,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CFProductCatalog" displayName="CFProductCatalog" ref="A4:J36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:J36"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CFProductCatalog" displayName="CFProductCatalog" ref="A4:J34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:J34"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="型号&#10;Model"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -512,7 +512,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>公开采购规格表 | 32 个 CF 型号 | 尺寸与穴盘适配请在打样前按图纸或实物复核 | Updated 2026-09-01</x:v>
+        <x:v>公开采购规格表 | 30 个 CF 型号 | 尺寸与穴盘适配请在打样前按图纸或实物复核 | Updated 2026-09-01</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -630,729 +630,729 @@
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="34" t="str">
-        <x:v>CF-004</x:v>
+        <x:v>CF-005</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>多肉育苗块 3.7 cm</x:v>
+        <x:v>扦插育苗块 5.0 cm</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>Succulent Starter Plug 3.7 cm</x:v>
+        <x:v>Cuttings Propagation Plug 5.0 cm</x:v>
       </x:c>
       <x:c r="D7" s="17" t="str">
-        <x:v>多肉育苗块 / Succulent Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E7" s="17" t="str">
-        <x:v>Top 3.3 cm / Bottom 2.8 cm / Height 3.7 cm</x:v>
+        <x:v>Top Ø 2.6 cm / Bottom Ø 1.6 cm / Height 5.0 cm</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>Succulent trays, 12-cell or 24-cell nursery boxes with opening ≥ 3.3 cm</x:v>
+        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
-        <x:v>Succulent propagation, small decorative planters and retail-ready planting sets</x:v>
+        <x:v>Cuttings propagation and narrow, deep propagation cells</x:v>
       </x:c>
       <x:c r="H7" s="17" t="str">
-        <x:v>300–500 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>600–900 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I7" s="17" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J7" s="17" t="str">
-        <x:v>assets/products/CF-004.jpg</x:v>
+        <x:v>assets/products/CF-005-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="36" t="str">
-        <x:v>CF-005</x:v>
+        <x:v>CF-006</x:v>
       </x:c>
       <x:c r="B8" s="37" t="str">
-        <x:v>扦插育苗块 5.0 cm</x:v>
+        <x:v>扦插育苗块 4.1 cm</x:v>
       </x:c>
       <x:c r="C8" s="37" t="str">
-        <x:v>Cuttings Propagation Plug 5.0 cm</x:v>
+        <x:v>Cuttings Propagation Plug 4.1 cm</x:v>
       </x:c>
       <x:c r="D8" s="37" t="str">
         <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E8" s="37" t="str">
-        <x:v>Top Ø 2.6 cm / Bottom Ø 1.6 cm / Height 5.0 cm</x:v>
+        <x:v>Top Ø 3.2 cm / Bottom Ø 2.2 cm / Height 4.1 cm</x:v>
       </x:c>
       <x:c r="F8" s="37" t="str">
         <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
       </x:c>
       <x:c r="G8" s="37" t="str">
-        <x:v>Cuttings propagation and narrow, deep propagation cells</x:v>
+        <x:v>Cuttings propagation and general nursery tray-fit trials</x:v>
       </x:c>
       <x:c r="H8" s="37" t="str">
-        <x:v>600–900 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>700–1000 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I8" s="37" t="str">
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J8" s="37" t="str">
-        <x:v>assets/products/CF-005-factory.webp</x:v>
+        <x:v>assets/products/CF-006-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="34" t="str">
-        <x:v>CF-006</x:v>
+        <x:v>CF-015</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>扦插育苗块 4.1 cm</x:v>
+        <x:v>兰花育苗块 4.5 cm</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
-        <x:v>Cuttings Propagation Plug 4.1 cm</x:v>
+        <x:v>Orchid Plug 4.5 cm</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>兰花基质块 / Orchid Plug</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
-        <x:v>Top Ø 3.2 cm / Bottom Ø 2.2 cm / Height 4.1 cm</x:v>
+        <x:v>Top 4.5 cm / Bottom 3.2 cm / Height 4.5 cm</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
+        <x:v>60-cell orchid trays</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
-        <x:v>Cuttings propagation and general nursery tray-fit trials</x:v>
+        <x:v>Orchid seedling production and stage-based transplant planning</x:v>
       </x:c>
       <x:c r="H9" s="17" t="str">
-        <x:v>700–1000 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>300–500 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I9" s="17" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J9" s="17" t="str">
-        <x:v>assets/products/CF-006-factory.webp</x:v>
+        <x:v>assets/products/CF-015.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="36" t="str">
-        <x:v>CF-010</x:v>
+        <x:v>CF-017</x:v>
       </x:c>
       <x:c r="B10" s="37" t="str">
-        <x:v>通用育苗块 4.1 cm</x:v>
+        <x:v>兰花基质块 5.3 cm</x:v>
       </x:c>
       <x:c r="C10" s="37" t="str">
-        <x:v>Universal Seedling Plug 4.1 cm</x:v>
+        <x:v>Orchid Plug 5.3 cm</x:v>
       </x:c>
       <x:c r="D10" s="37" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
+        <x:v>兰花基质块 / Orchid Plug</x:v>
       </x:c>
       <x:c r="E10" s="37" t="str">
-        <x:v>Top 3.2 cm / Bottom 2.2 cm / Height 4.1 cm</x:v>
+        <x:v>Top 5.3 cm / Bottom 3.4 cm / Height 4.8 cm</x:v>
       </x:c>
       <x:c r="F10" s="37" t="str">
-        <x:v>50–72-cell general seedling trays with approximately 3.2 cm openings</x:v>
+        <x:v>50-cell orchid or tissue-culture transition tray</x:v>
       </x:c>
       <x:c r="G10" s="37" t="str">
-        <x:v>General seed starting, cuttings and trial propagation programs</x:v>
+        <x:v>Young orchid plants, tissue-culture transition and early transplanting</x:v>
       </x:c>
       <x:c r="H10" s="37" t="str">
-        <x:v>1000–1500 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>200–300 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I10" s="37" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J10" s="37" t="str">
-        <x:v>assets/products/CF-010.jpg</x:v>
+        <x:v>assets/products/CF-017.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="34" t="str">
-        <x:v>CF-015</x:v>
+        <x:v>CF-025</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>兰花育苗块 4.5 cm</x:v>
+        <x:v>兰花种植杯 6.5 cm</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>Orchid Plug 4.5 cm</x:v>
+        <x:v>Orchid Planting Cup 6.5 cm</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str">
-        <x:v>兰花基质块 / Orchid Plug</x:v>
+        <x:v>兰花种植杯 / Orchid Planting Cup</x:v>
       </x:c>
       <x:c r="E11" s="17" t="str">
-        <x:v>Top 4.5 cm / Bottom 3.2 cm / Height 4.5 cm</x:v>
+        <x:v>Top 6.5 cm / Bottom 5.0 cm / Height 7.0 cm</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
-        <x:v>60-cell orchid trays</x:v>
+        <x:v>Orchid pots or 15–21-cell large planting trays</x:v>
       </x:c>
       <x:c r="G11" s="17" t="str">
-        <x:v>Orchid seedling production and stage-based transplant planning</x:v>
+        <x:v>Mid-stage orchid growth and transplanting into larger containers</x:v>
       </x:c>
       <x:c r="H11" s="17" t="str">
-        <x:v>300–500 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>120–180 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I11" s="17" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J11" s="17" t="str">
-        <x:v>assets/products/CF-015.jpg</x:v>
+        <x:v>assets/products/CF-025.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="36" t="str">
-        <x:v>CF-017</x:v>
+        <x:v>CF-028</x:v>
       </x:c>
       <x:c r="B12" s="37" t="str">
-        <x:v>兰花基质块 5.3 cm</x:v>
+        <x:v>高型兰花种植杯 8.3 cm</x:v>
       </x:c>
       <x:c r="C12" s="37" t="str">
-        <x:v>Orchid Plug 5.3 cm</x:v>
+        <x:v>Tall Orchid Cup 8.3 cm</x:v>
       </x:c>
       <x:c r="D12" s="37" t="str">
-        <x:v>兰花基质块 / Orchid Plug</x:v>
+        <x:v>兰花种植杯 / Orchid Planting Cup</x:v>
       </x:c>
       <x:c r="E12" s="37" t="str">
-        <x:v>Top 5.3 cm / Bottom 3.4 cm / Height 4.8 cm</x:v>
+        <x:v>Top 8.3 cm / Bottom 5.0 cm / Height 8.3 cm</x:v>
       </x:c>
       <x:c r="F12" s="37" t="str">
-        <x:v>50-cell orchid or tissue-culture transition tray</x:v>
+        <x:v>Orchid pots or 12–15-cell planting trays</x:v>
       </x:c>
       <x:c r="G12" s="37" t="str">
-        <x:v>Young orchid plants, tissue-culture transition and early transplanting</x:v>
+        <x:v>Tall orchid cultivation, specialty transplanting and larger plant stages</x:v>
       </x:c>
       <x:c r="H12" s="37" t="str">
-        <x:v>200–300 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>100–140 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I12" s="37" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J12" s="37" t="str">
-        <x:v>assets/products/CF-017.jpg</x:v>
+        <x:v>assets/products/CF-028.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="34" t="str">
-        <x:v>CF-025</x:v>
+        <x:v>CF-035</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>兰花种植杯 6.5 cm</x:v>
+        <x:v>大型兰花种植杯 10.5 cm</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>Orchid Planting Cup 6.5 cm</x:v>
+        <x:v>Tall Orchid Cup 10.5 cm</x:v>
       </x:c>
       <x:c r="D13" s="17" t="str">
         <x:v>兰花种植杯 / Orchid Planting Cup</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
-        <x:v>Top 6.5 cm / Bottom 5.0 cm / Height 7.0 cm</x:v>
+        <x:v>Top 10.5 cm / Bottom 7.0 cm / Height 10.5 cm</x:v>
       </x:c>
       <x:c r="F13" s="17" t="str">
-        <x:v>Orchid pots or 15–21-cell large planting trays</x:v>
+        <x:v>Orchid pots or 6–12-cell planting trays</x:v>
       </x:c>
       <x:c r="G13" s="17" t="str">
-        <x:v>Mid-stage orchid growth and transplanting into larger containers</x:v>
+        <x:v>Large orchid plants and premium transplanting formats</x:v>
       </x:c>
       <x:c r="H13" s="17" t="str">
-        <x:v>120–180 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>80–120 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I13" s="17" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J13" s="17" t="str">
-        <x:v>assets/products/CF-025.jpg</x:v>
+        <x:v>assets/products/CF-035.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="36" t="str">
-        <x:v>CF-028</x:v>
+        <x:v>CF-060</x:v>
       </x:c>
       <x:c r="B14" s="37" t="str">
-        <x:v>高型兰花种植杯 8.3 cm</x:v>
+        <x:v>60 穴蝴蝶兰育苗块 4.8 cm</x:v>
       </x:c>
       <x:c r="C14" s="37" t="str">
-        <x:v>Tall Orchid Cup 8.3 cm</x:v>
+        <x:v>Orchid Propagation Plug 4.8 cm</x:v>
       </x:c>
       <x:c r="D14" s="37" t="str">
-        <x:v>兰花种植杯 / Orchid Planting Cup</x:v>
+        <x:v>兰花基质块 / Orchid Plug</x:v>
       </x:c>
       <x:c r="E14" s="37" t="str">
-        <x:v>Top 8.3 cm / Bottom 5.0 cm / Height 8.3 cm</x:v>
+        <x:v>Top Ø 4.8 cm / Bottom Ø 3.4 cm / Height 4.6 cm</x:v>
       </x:c>
       <x:c r="F14" s="37" t="str">
-        <x:v>Orchid pots or 12–15-cell planting trays</x:v>
+        <x:v>60-cell orchid propagation tray</x:v>
       </x:c>
       <x:c r="G14" s="37" t="str">
-        <x:v>Tall orchid cultivation, specialty transplanting and larger plant stages</x:v>
+        <x:v>Professional Phalaenopsis propagation and tray-based nursery handling</x:v>
       </x:c>
       <x:c r="H14" s="37" t="str">
-        <x:v>100–140 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>Confirm after size option, carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I14" s="37" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J14" s="37" t="str">
-        <x:v>assets/products/CF-028.jpg</x:v>
+        <x:v>assets/products/CF-060-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="34" t="str">
-        <x:v>CF-035</x:v>
+        <x:v>CF-060B</x:v>
       </x:c>
       <x:c r="B15" s="17" t="str">
-        <x:v>大型兰花种植杯 10.5 cm</x:v>
+        <x:v>60 穴蝴蝶兰育苗块 5.2 cm</x:v>
       </x:c>
       <x:c r="C15" s="17" t="str">
-        <x:v>Tall Orchid Cup 10.5 cm</x:v>
+        <x:v>Orchid Propagation Plug 5.2 cm</x:v>
       </x:c>
       <x:c r="D15" s="17" t="str">
-        <x:v>兰花种植杯 / Orchid Planting Cup</x:v>
+        <x:v>兰花基质块 / Orchid Plug</x:v>
       </x:c>
       <x:c r="E15" s="17" t="str">
-        <x:v>Top 10.5 cm / Bottom 7.0 cm / Height 10.5 cm</x:v>
+        <x:v>Top Ø 5.2 cm / Bottom Ø 3.8 cm / Height 4.8 cm</x:v>
       </x:c>
       <x:c r="F15" s="17" t="str">
-        <x:v>Orchid pots or 6–12-cell planting trays</x:v>
+        <x:v>60-cell orchid propagation tray</x:v>
       </x:c>
       <x:c r="G15" s="17" t="str">
-        <x:v>Large orchid plants and premium transplanting formats</x:v>
+        <x:v>Professional Phalaenopsis propagation requiring a larger plug volume</x:v>
       </x:c>
       <x:c r="H15" s="17" t="str">
-        <x:v>80–120 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>Confirm after size option, carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I15" s="17" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J15" s="17" t="str">
-        <x:v>assets/products/CF-035.jpg</x:v>
+        <x:v>assets/products/CF-060B-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="36" t="str">
-        <x:v>CF-060</x:v>
+        <x:v>CF-067</x:v>
       </x:c>
       <x:c r="B16" s="37" t="str">
-        <x:v>60 穴蝴蝶兰育苗块 4.8 cm</x:v>
+        <x:v>多肉种植杯 6.7 cm</x:v>
       </x:c>
       <x:c r="C16" s="37" t="str">
-        <x:v>Orchid Propagation Plug 4.8 cm</x:v>
+        <x:v>Succulent Growing Cup 6.7 cm</x:v>
       </x:c>
       <x:c r="D16" s="37" t="str">
-        <x:v>兰花基质块 / Orchid Plug</x:v>
+        <x:v>多肉种植杯 / Succulent Growing Cup</x:v>
       </x:c>
       <x:c r="E16" s="37" t="str">
-        <x:v>Top Ø 4.8 cm / Bottom Ø 3.4 cm / Height 4.6 cm</x:v>
+        <x:v>Top 6.7 cm / Bottom 4.8 cm / Height 6.5 cm</x:v>
       </x:c>
       <x:c r="F16" s="37" t="str">
-        <x:v>60-cell orchid propagation tray</x:v>
+        <x:v>6.7 cm pot holders, succulent cup display trays or decorative planters</x:v>
       </x:c>
       <x:c r="G16" s="37" t="str">
-        <x:v>Professional Phalaenopsis propagation and tray-based nursery handling</x:v>
+        <x:v>Succulent planting, decorative cup planting and home-garden retail sets</x:v>
       </x:c>
       <x:c r="H16" s="37" t="str">
-        <x:v>Confirm after size option, carton size and packaging format are approved.</x:v>
+        <x:v>120–200 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I16" s="37" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J16" s="37" t="str">
-        <x:v>assets/products/CF-060-factory.webp</x:v>
+        <x:v>assets/products/CF-067.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="34" t="str">
-        <x:v>CF-060B</x:v>
+        <x:v>CF-072</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>60 穴蝴蝶兰育苗块 5.2 cm</x:v>
+        <x:v>72 穴组培育苗块 4.0 cm</x:v>
       </x:c>
       <x:c r="C17" s="17" t="str">
-        <x:v>Orchid Propagation Plug 5.2 cm</x:v>
+        <x:v>Tissue Culture Propagation Plug 4.0 cm</x:v>
       </x:c>
       <x:c r="D17" s="17" t="str">
-        <x:v>兰花基质块 / Orchid Plug</x:v>
+        <x:v>组培基质块 / Tissue Culture Plug</x:v>
       </x:c>
       <x:c r="E17" s="17" t="str">
-        <x:v>Top Ø 5.2 cm / Bottom Ø 3.8 cm / Height 4.8 cm</x:v>
+        <x:v>Top Ø 4.0 cm / Bottom Ø 2.0 cm / Height 4.0 cm</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>60-cell orchid propagation tray</x:v>
+        <x:v>72-cell propagation tray</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>Professional Phalaenopsis propagation and tray-based nursery handling</x:v>
+        <x:v>Tissue-culture acclimatization and nursery transition in 72-cell trays</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
-        <x:v>Confirm after size option, carton size and packaging format are approved.</x:v>
+        <x:v>72 plugs / tray × 24 trays / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I17" s="17" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J17" s="17" t="str">
-        <x:v>assets/products/CF-060B-factory.webp</x:v>
+        <x:v>assets/products/CF-072-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="36" t="str">
-        <x:v>CF-067</x:v>
+        <x:v>CF-104</x:v>
       </x:c>
       <x:c r="B18" s="37" t="str">
-        <x:v>多肉种植杯 6.7 cm</x:v>
+        <x:v>通用育苗块 4.0 cm</x:v>
       </x:c>
       <x:c r="C18" s="37" t="str">
-        <x:v>Succulent Growing Cup 6.7 cm</x:v>
+        <x:v>Nursery Plug 4.0 cm</x:v>
       </x:c>
       <x:c r="D18" s="37" t="str">
-        <x:v>多肉种植杯 / Succulent Growing Cup</x:v>
+        <x:v>育苗基质块 / Seedling Plug</x:v>
       </x:c>
       <x:c r="E18" s="37" t="str">
-        <x:v>Top 6.7 cm / Bottom 4.8 cm / Height 6.5 cm</x:v>
+        <x:v>Top Ø 3.1 cm / Bottom Ø 2.5 cm / Height 4.0 cm</x:v>
       </x:c>
       <x:c r="F18" s="37" t="str">
-        <x:v>6.7 cm pot holders, succulent cup display trays or decorative planters</x:v>
+        <x:v>Nursery and propagation trays with approximately 3.1 cm openings</x:v>
       </x:c>
       <x:c r="G18" s="37" t="str">
-        <x:v>Succulent planting, decorative cup planting and home-garden retail sets</x:v>
+        <x:v>General nursery propagation, seed starting and transplant trials</x:v>
       </x:c>
       <x:c r="H18" s="37" t="str">
-        <x:v>120–200 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I18" s="37" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J18" s="37" t="str">
-        <x:v>assets/products/CF-067.jpg</x:v>
+        <x:v>assets/products/CF-104.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="A19" s="34" t="str">
-        <x:v>CF-072</x:v>
+        <x:v>CF-128</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>72 穴组培育苗块 4.0 cm</x:v>
+        <x:v>128 穴组培育苗块 3.8 cm</x:v>
       </x:c>
       <x:c r="C19" s="17" t="str">
-        <x:v>Tissue Culture Propagation Plug 4.0 cm</x:v>
+        <x:v>Tissue Culture Propagation Plug 3.8 cm</x:v>
       </x:c>
       <x:c r="D19" s="17" t="str">
         <x:v>组培基质块 / Tissue Culture Plug</x:v>
       </x:c>
       <x:c r="E19" s="17" t="str">
-        <x:v>Top Ø 4.0 cm / Bottom Ø 2.0 cm / Height 4.0 cm</x:v>
+        <x:v>Top Ø 3.0 cm / Bottom Ø 1.4 cm / Height 3.8 cm</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
-        <x:v>72-cell propagation tray</x:v>
+        <x:v>128-cell propagation tray</x:v>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>Tissue-culture acclimatization and nursery transition in 72-cell trays</x:v>
+        <x:v>Tissue-culture acclimatization and compact nursery propagation</x:v>
       </x:c>
       <x:c r="H19" s="17" t="str">
-        <x:v>72 plugs / tray × 24 trays / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>128 plugs / sheet × 20 sheets / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I19" s="17" t="str">
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J19" s="17" t="str">
-        <x:v>assets/products/CF-072-factory.webp</x:v>
+        <x:v>assets/products/CF-128-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="46" customHeight="1">
       <x:c r="A20" s="36" t="str">
-        <x:v>CF-104</x:v>
+        <x:v>CF-128B</x:v>
       </x:c>
       <x:c r="B20" s="37" t="str">
-        <x:v>通用育苗块 4.0 cm</x:v>
+        <x:v>128 穴扦插育苗块 3.8 cm</x:v>
       </x:c>
       <x:c r="C20" s="37" t="str">
-        <x:v>Nursery Plug 4.0 cm</x:v>
+        <x:v>128-Cell Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="D20" s="37" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E20" s="37" t="str">
-        <x:v>Top Ø 3.1 cm / Bottom Ø 2.5 cm / Height 4.0 cm</x:v>
+        <x:v>Top Ø 3.0 cm / Bottom Ø 1.4 cm / Height 3.8 cm</x:v>
       </x:c>
       <x:c r="F20" s="37" t="str">
-        <x:v>Nursery and propagation trays with approximately 3.1 cm openings</x:v>
+        <x:v>128-cell cuttings propagation tray</x:v>
       </x:c>
       <x:c r="G20" s="37" t="str">
-        <x:v>General nursery propagation, seed starting and transplant trials</x:v>
+        <x:v>High-density cuttings propagation in 128-cell trays</x:v>
       </x:c>
       <x:c r="H20" s="37" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
+        <x:v>128 plugs / sheet × 20 sheets / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I20" s="37" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J20" s="37" t="str">
-        <x:v>assets/products/CF-104.webp</x:v>
+        <x:v>assets/products/CF-128B-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="46" customHeight="1">
       <x:c r="A21" s="34" t="str">
-        <x:v>CF-128</x:v>
+        <x:v>CF-129</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>128 穴组培育苗块 3.8 cm</x:v>
+        <x:v>圆柱形育苗块 3.1 cm</x:v>
       </x:c>
       <x:c r="C21" s="17" t="str">
-        <x:v>Tissue Culture Propagation Plug 3.8 cm</x:v>
+        <x:v>Cylindrical Plug 3.1 cm</x:v>
       </x:c>
       <x:c r="D21" s="17" t="str">
-        <x:v>组培基质块 / Tissue Culture Plug</x:v>
+        <x:v>圆柱形基质块 / Cylindrical Plug</x:v>
       </x:c>
       <x:c r="E21" s="17" t="str">
-        <x:v>Top Ø 3.0 cm / Bottom Ø 1.4 cm / Height 3.8 cm</x:v>
+        <x:v>Top 2.6 cm / Bottom 2.3 cm / Height 3.1 cm</x:v>
       </x:c>
       <x:c r="F21" s="17" t="str">
-        <x:v>128-cell propagation tray</x:v>
+        <x:v>105-cell or 128-cell propagation trays</x:v>
       </x:c>
       <x:c r="G21" s="17" t="str">
-        <x:v>Tissue-culture acclimatization and compact nursery propagation</x:v>
+        <x:v>Cuttings, seed starting and cylindrical cavity applications</x:v>
       </x:c>
       <x:c r="H21" s="17" t="str">
-        <x:v>128 plugs / sheet × 20 sheets / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>800–1200 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I21" s="17" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J21" s="17" t="str">
-        <x:v>assets/products/CF-128-factory.webp</x:v>
+        <x:v>assets/products/CF-129.png</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="46" customHeight="1">
       <x:c r="A22" s="36" t="str">
-        <x:v>CF-128B</x:v>
+        <x:v>CF-167</x:v>
       </x:c>
       <x:c r="B22" s="37" t="str">
-        <x:v>128 穴扦插育苗块 3.8 cm</x:v>
+        <x:v>紧凑型扦插育苗块 3.0 cm</x:v>
       </x:c>
       <x:c r="C22" s="37" t="str">
-        <x:v>128-Cell Cuttings Propagation Plug</x:v>
+        <x:v>Compact Cuttings Plug 3.0 cm</x:v>
       </x:c>
       <x:c r="D22" s="37" t="str">
         <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E22" s="37" t="str">
-        <x:v>Top Ø 3.0 cm / Bottom Ø 1.4 cm / Height 3.8 cm</x:v>
+        <x:v>Top Ø 2.5 cm / Bottom Ø 2.1 cm / Height 3.0 cm</x:v>
       </x:c>
       <x:c r="F22" s="37" t="str">
-        <x:v>128-cell cuttings propagation tray</x:v>
+        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
       </x:c>
       <x:c r="G22" s="37" t="str">
-        <x:v>High-density cuttings propagation in 128-cell trays</x:v>
+        <x:v>High-density cuttings propagation and compact nursery cells</x:v>
       </x:c>
       <x:c r="H22" s="37" t="str">
-        <x:v>128 plugs / sheet × 20 sheets / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I22" s="37" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J22" s="37" t="str">
-        <x:v>assets/products/CF-128B-factory.webp</x:v>
+        <x:v>assets/products/CF-167-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="46" customHeight="1">
       <x:c r="A23" s="34" t="str">
-        <x:v>CF-129</x:v>
+        <x:v>CF-200</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
-        <x:v>圆柱形育苗块 3.1 cm</x:v>
+        <x:v>200 穴扦插育苗块 2.8 cm</x:v>
       </x:c>
       <x:c r="C23" s="17" t="str">
-        <x:v>Cylindrical Plug 3.1 cm</x:v>
+        <x:v>200-Cell Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="D23" s="17" t="str">
-        <x:v>圆柱形基质块 / Cylindrical Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E23" s="17" t="str">
-        <x:v>Top 2.6 cm / Bottom 2.3 cm / Height 3.1 cm</x:v>
+        <x:v>Top Ø 2.3 cm / Bottom Ø 2.0 cm / Height 2.8 cm</x:v>
       </x:c>
       <x:c r="F23" s="17" t="str">
-        <x:v>105-cell or 128-cell propagation trays</x:v>
+        <x:v>200-cell propagation tray</x:v>
       </x:c>
       <x:c r="G23" s="17" t="str">
-        <x:v>Cuttings, seed starting and cylindrical cavity applications</x:v>
+        <x:v>High-density cuttings propagation and automated 200-cell nursery workflows</x:v>
       </x:c>
       <x:c r="H23" s="17" t="str">
-        <x:v>800–1200 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>200 plugs / tray × 10 trays / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I23" s="17" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J23" s="17" t="str">
-        <x:v>assets/products/CF-129.png</x:v>
+        <x:v>assets/products/CF-200-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="46" customHeight="1">
       <x:c r="A24" s="36" t="str">
-        <x:v>CF-167</x:v>
+        <x:v>CF-901</x:v>
       </x:c>
       <x:c r="B24" s="37" t="str">
-        <x:v>紧凑型扦插育苗块 3.0 cm</x:v>
+        <x:v>鹿角蕨上板球 20 cm</x:v>
       </x:c>
       <x:c r="C24" s="37" t="str">
-        <x:v>Compact Cuttings Plug 3.0 cm</x:v>
+        <x:v>Staghorn Fern Mounting Ball 20 cm</x:v>
       </x:c>
       <x:c r="D24" s="37" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>鹿角蕨上板球 / Staghorn Fern Mounting Ball</x:v>
       </x:c>
       <x:c r="E24" s="37" t="str">
-        <x:v>Top Ø 2.5 cm / Bottom Ø 2.1 cm / Height 3.0 cm</x:v>
+        <x:v>Diameter 20 cm / Height 10 cm / Center hole 9.5 cm</x:v>
       </x:c>
       <x:c r="F24" s="37" t="str">
-        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
+        <x:v>Staghorn fern mounting boards, hanging displays or epiphyte mounting systems</x:v>
       </x:c>
       <x:c r="G24" s="37" t="str">
-        <x:v>High-density cuttings propagation and compact nursery cells</x:v>
+        <x:v>Large staghorn fern board-mounting trials and decorative epiphyte displays</x:v>
       </x:c>
       <x:c r="H24" s="37" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
+        <x:v>20–40 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I24" s="37" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J24" s="37" t="str">
-        <x:v>assets/products/CF-167-factory.webp</x:v>
+        <x:v>assets/products/CF-901.png</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="46" customHeight="1">
       <x:c r="A25" s="34" t="str">
-        <x:v>CF-200</x:v>
+        <x:v>CF-902</x:v>
       </x:c>
       <x:c r="B25" s="17" t="str">
-        <x:v>200 穴扦插育苗块 2.8 cm</x:v>
+        <x:v>鹿角蕨上板球 16 cm</x:v>
       </x:c>
       <x:c r="C25" s="17" t="str">
-        <x:v>200-Cell Cuttings Propagation Plug</x:v>
+        <x:v>Staghorn Fern Mounting Ball 16 cm</x:v>
       </x:c>
       <x:c r="D25" s="17" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>鹿角蕨上板球 / Staghorn Fern Mounting Ball</x:v>
       </x:c>
       <x:c r="E25" s="17" t="str">
-        <x:v>Top Ø 2.3 cm / Bottom Ø 2.0 cm / Height 2.8 cm</x:v>
+        <x:v>Diameter 16 cm / Height 8 cm / Center hole 8.2 cm</x:v>
       </x:c>
       <x:c r="F25" s="17" t="str">
-        <x:v>200-cell propagation tray</x:v>
+        <x:v>Staghorn fern mounting boards, hanging displays or epiphyte mounting systems</x:v>
       </x:c>
       <x:c r="G25" s="17" t="str">
-        <x:v>High-density cuttings propagation and automated 200-cell nursery workflows</x:v>
+        <x:v>Medium staghorn fern board-mounting trials and retail epiphyte displays</x:v>
       </x:c>
       <x:c r="H25" s="17" t="str">
-        <x:v>200 plugs / tray × 10 trays / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>30–60 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I25" s="17" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J25" s="17" t="str">
-        <x:v>assets/products/CF-200-factory.webp</x:v>
+        <x:v>assets/products/CF-902.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="46" customHeight="1">
       <x:c r="A26" s="36" t="str">
-        <x:v>CF-901</x:v>
+        <x:v>CF-903</x:v>
       </x:c>
       <x:c r="B26" s="37" t="str">
-        <x:v>鹿角蕨上板球 20 cm</x:v>
+        <x:v>鹿角蕨上板球 11 cm</x:v>
       </x:c>
       <x:c r="C26" s="37" t="str">
-        <x:v>Staghorn Fern Mounting Ball 20 cm</x:v>
+        <x:v>Staghorn Fern Mounting Ball 11 cm</x:v>
       </x:c>
       <x:c r="D26" s="37" t="str">
         <x:v>鹿角蕨上板球 / Staghorn Fern Mounting Ball</x:v>
       </x:c>
       <x:c r="E26" s="37" t="str">
-        <x:v>Diameter 20 cm / Height 10 cm / Center hole 9.5 cm</x:v>
+        <x:v>Diameter 11 cm / Height 5.5 cm / Center hole 5.5 cm</x:v>
       </x:c>
       <x:c r="F26" s="37" t="str">
         <x:v>Staghorn fern mounting boards, hanging displays or epiphyte mounting systems</x:v>
       </x:c>
       <x:c r="G26" s="37" t="str">
-        <x:v>Large staghorn fern board-mounting trials and decorative epiphyte displays</x:v>
+        <x:v>Compact staghorn fern board-mounting trials and small epiphyte displays</x:v>
       </x:c>
       <x:c r="H26" s="37" t="str">
-        <x:v>20–40 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>60–100 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
       </x:c>
       <x:c r="I26" s="37" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J26" s="37" t="str">
-        <x:v>assets/products/CF-901.png</x:v>
+        <x:v>assets/products/CF-903.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="46" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>CF-902</x:v>
+        <x:v>CF-2735</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>鹿角蕨上板球 16 cm</x:v>
+        <x:v>紧凑型组培基质块 3.5 cm</x:v>
       </x:c>
       <x:c r="C27" s="17" t="str">
-        <x:v>Staghorn Fern Mounting Ball 16 cm</x:v>
+        <x:v>Tissue Culture Propagation Plug 3.5 cm</x:v>
       </x:c>
       <x:c r="D27" s="17" t="str">
-        <x:v>鹿角蕨上板球 / Staghorn Fern Mounting Ball</x:v>
+        <x:v>组培基质块 / Tissue Culture Plug</x:v>
       </x:c>
       <x:c r="E27" s="17" t="str">
-        <x:v>Diameter 16 cm / Height 8 cm / Center hole 8.2 cm</x:v>
+        <x:v>Top Ø 2.7 cm / Bottom Ø 2.3 cm / Height 3.5 cm</x:v>
       </x:c>
       <x:c r="F27" s="17" t="str">
-        <x:v>Staghorn fern mounting boards, hanging displays or epiphyte mounting systems</x:v>
+        <x:v>180-cell propagation tray</x:v>
       </x:c>
       <x:c r="G27" s="17" t="str">
-        <x:v>Medium staghorn fern board-mounting trials and retail epiphyte displays</x:v>
+        <x:v>Tissue-culture acclimatization and compact high-count trays</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
-        <x:v>30–60 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I27" s="17" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J27" s="17" t="str">
-        <x:v>assets/products/CF-902.jpg</x:v>
+        <x:v>assets/products/CF-2735-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="46" customHeight="1">
       <x:c r="A28" s="36" t="str">
-        <x:v>CF-903</x:v>
+        <x:v>CF-3038</x:v>
       </x:c>
       <x:c r="B28" s="37" t="str">
-        <x:v>鹿角蕨上板球 11 cm</x:v>
+        <x:v>扦插育苗块 3.8 cm</x:v>
       </x:c>
       <x:c r="C28" s="37" t="str">
-        <x:v>Staghorn Fern Mounting Ball 11 cm</x:v>
+        <x:v>Cuttings Propagation Plug 3.8 cm</x:v>
       </x:c>
       <x:c r="D28" s="37" t="str">
-        <x:v>鹿角蕨上板球 / Staghorn Fern Mounting Ball</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E28" s="37" t="str">
-        <x:v>Diameter 11 cm / Height 5.5 cm / Center hole 5.5 cm</x:v>
+        <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
       </x:c>
       <x:c r="F28" s="37" t="str">
-        <x:v>Staghorn fern mounting boards, hanging displays or epiphyte mounting systems</x:v>
+        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
       </x:c>
       <x:c r="G28" s="37" t="str">
-        <x:v>Compact staghorn fern board-mounting trials and small epiphyte displays</x:v>
+        <x:v>Commercial cuttings propagation and model-to-tray trials</x:v>
       </x:c>
       <x:c r="H28" s="37" t="str">
-        <x:v>60–100 pcs / carton (reference; final count varies by carton size and packaging format)</x:v>
+        <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I28" s="37" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J28" s="37" t="str">
-        <x:v>assets/products/CF-903.jpg</x:v>
+        <x:v>assets/products/CF-3038-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="46" customHeight="1">
       <x:c r="A29" s="34" t="str">
-        <x:v>CF-2735</x:v>
+        <x:v>CF-3038B</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>紧凑型组培基质块 3.5 cm</x:v>
+        <x:v>水培育苗块 3.8 cm B 型</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
-        <x:v>Tissue Culture Propagation Plug 3.5 cm</x:v>
+        <x:v>Hydroponic Propagation Plug 3.8 cm</x:v>
       </x:c>
       <x:c r="D29" s="17" t="str">
-        <x:v>组培基质块 / Tissue Culture Plug</x:v>
+        <x:v>水培育苗块 / Hydroponic Plug</x:v>
       </x:c>
       <x:c r="E29" s="17" t="str">
-        <x:v>Top Ø 2.7 cm / Bottom Ø 2.3 cm / Height 3.5 cm</x:v>
+        <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
       </x:c>
       <x:c r="F29" s="17" t="str">
-        <x:v>180-cell propagation tray</x:v>
+        <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
       </x:c>
       <x:c r="G29" s="17" t="str">
-        <x:v>Tissue-culture acclimatization and compact high-count trays</x:v>
+        <x:v>Hydroponic sowing, nursery production and controlled-environment systems</x:v>
       </x:c>
       <x:c r="H29" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1361,30 +1361,30 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J29" s="17" t="str">
-        <x:v>assets/products/CF-2735-factory.webp</x:v>
+        <x:v>assets/products/CF-3038B-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="46" customHeight="1">
       <x:c r="A30" s="36" t="str">
-        <x:v>CF-3038</x:v>
+        <x:v>CF-3240</x:v>
       </x:c>
       <x:c r="B30" s="37" t="str">
-        <x:v>扦插育苗块 3.8 cm</x:v>
+        <x:v>扦插育苗块 4.0 cm</x:v>
       </x:c>
       <x:c r="C30" s="37" t="str">
-        <x:v>Cuttings Propagation Plug 3.8 cm</x:v>
+        <x:v>Cuttings Propagation Plug 4.0 cm</x:v>
       </x:c>
       <x:c r="D30" s="37" t="str">
         <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E30" s="37" t="str">
-        <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
+        <x:v>Top Ø 3.2 cm / Bottom Ø 2.5 cm / Height 4.0 cm</x:v>
       </x:c>
       <x:c r="F30" s="37" t="str">
         <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
       </x:c>
       <x:c r="G30" s="37" t="str">
-        <x:v>Commercial cuttings propagation and model-to-tray trials</x:v>
+        <x:v>Cuttings propagation and tray-fit projects requiring a 3.2 cm top diameter</x:v>
       </x:c>
       <x:c r="H30" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1393,30 +1393,30 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J30" s="37" t="str">
-        <x:v>assets/products/CF-3038-factory.webp</x:v>
+        <x:v>assets/products/CF-3240-dimensions.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="46" customHeight="1">
       <x:c r="A31" s="34" t="str">
-        <x:v>CF-3038B</x:v>
+        <x:v>CF-3545</x:v>
       </x:c>
       <x:c r="B31" s="17" t="str">
-        <x:v>水培育苗块 3.8 cm B 型</x:v>
+        <x:v>水培育苗块 4.5 cm</x:v>
       </x:c>
       <x:c r="C31" s="17" t="str">
-        <x:v>Hydroponic Propagation Plug 3.8 cm</x:v>
+        <x:v>Hydroponic Propagation Plug 4.5 cm</x:v>
       </x:c>
       <x:c r="D31" s="17" t="str">
         <x:v>水培育苗块 / Hydroponic Plug</x:v>
       </x:c>
       <x:c r="E31" s="17" t="str">
-        <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
+        <x:v>Top Ø 3.5 cm / Bottom Ø 2.2 cm / Height 4.5 cm</x:v>
       </x:c>
       <x:c r="F31" s="17" t="str">
         <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
       </x:c>
       <x:c r="G31" s="17" t="str">
-        <x:v>Hydroponic sowing, nursery production and controlled-environment systems</x:v>
+        <x:v>Hydroponic propagation and controlled-environment nursery production</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1425,30 +1425,30 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J31" s="17" t="str">
-        <x:v>assets/products/CF-3038B-factory.webp</x:v>
+        <x:v>assets/products/CF-3545-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="46" customHeight="1">
       <x:c r="A32" s="36" t="str">
-        <x:v>CF-3240</x:v>
+        <x:v>CF-3550</x:v>
       </x:c>
       <x:c r="B32" s="37" t="str">
-        <x:v>扦插育苗块 4.0 cm</x:v>
+        <x:v>高型育苗块 5.3 cm</x:v>
       </x:c>
       <x:c r="C32" s="37" t="str">
-        <x:v>Cuttings Propagation Plug 4.0 cm</x:v>
+        <x:v>Tall Nursery Plug 5.3 cm</x:v>
       </x:c>
       <x:c r="D32" s="37" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>育苗基质块 / Seedling Plug</x:v>
       </x:c>
       <x:c r="E32" s="37" t="str">
-        <x:v>Top Ø 3.2 cm / Bottom Ø 2.5 cm / Height 4.0 cm</x:v>
+        <x:v>Top Ø 3.7 cm / Bottom Ø 2.2 cm / Height 5.3 cm</x:v>
       </x:c>
       <x:c r="F32" s="37" t="str">
-        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
+        <x:v>Deeper nursery and propagation trays with approximately 3.7 cm openings</x:v>
       </x:c>
       <x:c r="G32" s="37" t="str">
-        <x:v>Cuttings propagation and tray-fit projects requiring a 3.2 cm top diameter</x:v>
+        <x:v>Seedlings and cuttings requiring a taller propagation format</x:v>
       </x:c>
       <x:c r="H32" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1457,30 +1457,30 @@
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J32" s="37" t="str">
-        <x:v>assets/products/CF-3240-dimensions.webp</x:v>
+        <x:v>assets/products/CF-3550.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="46" customHeight="1">
       <x:c r="A33" s="34" t="str">
-        <x:v>CF-3545</x:v>
+        <x:v>CF-5050</x:v>
       </x:c>
       <x:c r="B33" s="17" t="str">
-        <x:v>水培育苗块 4.5 cm</x:v>
+        <x:v>50 穴扦插育苗块 5.0 cm</x:v>
       </x:c>
       <x:c r="C33" s="17" t="str">
-        <x:v>Hydroponic Propagation Plug 4.5 cm</x:v>
+        <x:v>50-Cell Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="D33" s="17" t="str">
-        <x:v>水培育苗块 / Hydroponic Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E33" s="17" t="str">
-        <x:v>Top Ø 3.5 cm / Bottom Ø 2.2 cm / Height 4.5 cm</x:v>
+        <x:v>Top Ø 5.0 cm / Bottom Ø 3.8 cm / Height 5.0 cm</x:v>
       </x:c>
       <x:c r="F33" s="17" t="str">
-        <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
+        <x:v>50-cell propagation tray</x:v>
       </x:c>
       <x:c r="G33" s="17" t="str">
-        <x:v>Hydroponic propagation and controlled-environment nursery production</x:v>
+        <x:v>Larger cuttings and commercial 50-cell nursery workflows</x:v>
       </x:c>
       <x:c r="H33" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1489,102 +1489,38 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J33" s="17" t="str">
-        <x:v>assets/products/CF-3545-factory.webp</x:v>
+        <x:v>assets/products/CF-5050-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="46" customHeight="1">
-      <x:c r="A34" s="36" t="str">
-        <x:v>CF-3550</x:v>
-      </x:c>
-      <x:c r="B34" s="37" t="str">
-        <x:v>高型育苗块 5.3 cm</x:v>
-      </x:c>
-      <x:c r="C34" s="37" t="str">
-        <x:v>Tall Nursery Plug 5.3 cm</x:v>
-      </x:c>
-      <x:c r="D34" s="37" t="str">
+      <x:c r="A34" s="38" t="str">
+        <x:v>CF-7050</x:v>
+      </x:c>
+      <x:c r="B34" s="39" t="str">
+        <x:v>高型育苗块 6.8 cm</x:v>
+      </x:c>
+      <x:c r="C34" s="39" t="str">
+        <x:v>Tall Nursery Plug 6.8 cm</x:v>
+      </x:c>
+      <x:c r="D34" s="39" t="str">
         <x:v>育苗基质块 / Seedling Plug</x:v>
       </x:c>
-      <x:c r="E34" s="37" t="str">
-        <x:v>Top Ø 3.7 cm / Bottom Ø 2.2 cm / Height 5.3 cm</x:v>
-      </x:c>
-      <x:c r="F34" s="37" t="str">
-        <x:v>Deeper nursery and propagation trays with approximately 3.7 cm openings</x:v>
-      </x:c>
-      <x:c r="G34" s="37" t="str">
-        <x:v>Seedlings and cuttings requiring a taller propagation format</x:v>
-      </x:c>
-      <x:c r="H34" s="37" t="str">
+      <x:c r="E34" s="39" t="str">
+        <x:v>Top Ø 4.8 cm / Bottom Ø 3.5 cm / Height 6.8 cm</x:v>
+      </x:c>
+      <x:c r="F34" s="39" t="str">
+        <x:v>Deep nursery trays, pots or holders with approximately 4.8 cm openings</x:v>
+      </x:c>
+      <x:c r="G34" s="39" t="str">
+        <x:v>Larger seedlings, deeper rooting stages and transplant programs</x:v>
+      </x:c>
+      <x:c r="H34" s="39" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
-      <x:c r="I34" s="37" t="str">
+      <x:c r="I34" s="39" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
-      <x:c r="J34" s="37" t="str">
-        <x:v>assets/products/CF-3550.webp</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="46" customHeight="1">
-      <x:c r="A35" s="34" t="str">
-        <x:v>CF-5050</x:v>
-      </x:c>
-      <x:c r="B35" s="17" t="str">
-        <x:v>50 穴扦插育苗块 5.0 cm</x:v>
-      </x:c>
-      <x:c r="C35" s="17" t="str">
-        <x:v>50-Cell Cuttings Propagation Plug</x:v>
-      </x:c>
-      <x:c r="D35" s="17" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
-      </x:c>
-      <x:c r="E35" s="17" t="str">
-        <x:v>Top Ø 5.0 cm / Bottom Ø 3.8 cm / Height 5.0 cm</x:v>
-      </x:c>
-      <x:c r="F35" s="17" t="str">
-        <x:v>50-cell propagation tray</x:v>
-      </x:c>
-      <x:c r="G35" s="17" t="str">
-        <x:v>Larger cuttings and commercial 50-cell nursery workflows</x:v>
-      </x:c>
-      <x:c r="H35" s="17" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
-      </x:c>
-      <x:c r="I35" s="17" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
-      </x:c>
-      <x:c r="J35" s="17" t="str">
-        <x:v>assets/products/CF-5050-factory.webp</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="46" customHeight="1">
-      <x:c r="A36" s="38" t="str">
-        <x:v>CF-7050</x:v>
-      </x:c>
-      <x:c r="B36" s="39" t="str">
-        <x:v>高型育苗块 6.8 cm</x:v>
-      </x:c>
-      <x:c r="C36" s="39" t="str">
-        <x:v>Tall Nursery Plug 6.8 cm</x:v>
-      </x:c>
-      <x:c r="D36" s="39" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
-      </x:c>
-      <x:c r="E36" s="39" t="str">
-        <x:v>Top Ø 4.8 cm / Bottom Ø 3.5 cm / Height 6.8 cm</x:v>
-      </x:c>
-      <x:c r="F36" s="39" t="str">
-        <x:v>Deep nursery trays, pots or holders with approximately 4.8 cm openings</x:v>
-      </x:c>
-      <x:c r="G36" s="39" t="str">
-        <x:v>Larger seedlings, deeper rooting stages and transplant programs</x:v>
-      </x:c>
-      <x:c r="H36" s="39" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
-      </x:c>
-      <x:c r="I36" s="39" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
-      </x:c>
-      <x:c r="J36" s="39" t="str">
+      <x:c r="J34" s="39" t="str">
         <x:v>assets/products/CF-7050.webp</x:v>
       </x:c>
     </x:row>
@@ -1595,7 +1531,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f2c560f40be443c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3decfa7730504456"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1631,7 +1567,7 @@
         <x:v>产品范围</x:v>
       </x:c>
       <x:c r="B4" s="43" t="str">
-        <x:v>32 个公开 CF 型号；不含工厂内部型号映射。</x:v>
+        <x:v>30 个公开 CF 型号；不含工厂内部型号映射。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">

</xml_diff>

<commit_message>
Clean product imagery and centralize silent factory videos
</commit_message>
<xml_diff>
--- a/docs/MCCS_CF_Product_Specifications.xlsx
+++ b/docs/MCCS_CF_Product_Specifications.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF 产品规格" sheetId="1" r:id="R38dba418bc9b43c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购说明" sheetId="2" r:id="R64c1203b4fd2442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF 产品规格" sheetId="1" r:id="R338186c641ff4d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购说明" sheetId="2" r:id="R74de7c8ad19a48ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -141,7 +141,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -236,12 +236,6 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -271,8 +265,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CFProductCatalog" displayName="CFProductCatalog" ref="A4:J34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:J34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CFProductCatalog" displayName="CFProductCatalog" ref="A4:J33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:J33"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="型号&#10;Model"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -512,7 +506,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>公开采购规格表 | 30 个 CF 型号 | 尺寸与穴盘适配请在打样前按图纸或实物复核 | Updated 2026-09-01</x:v>
+        <x:v>公开采购规格表 | 29 个 CF 型号 | 尺寸与穴盘适配请在打样前按图纸或实物复核 | Updated 2026-09-01</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1366,25 +1360,25 @@
     </x:row>
     <x:row r="30" ht="46" customHeight="1">
       <x:c r="A30" s="36" t="str">
-        <x:v>CF-3240</x:v>
+        <x:v>CF-3545</x:v>
       </x:c>
       <x:c r="B30" s="37" t="str">
-        <x:v>扦插育苗块 4.0 cm</x:v>
+        <x:v>水培育苗块 4.5 cm</x:v>
       </x:c>
       <x:c r="C30" s="37" t="str">
-        <x:v>Cuttings Propagation Plug 4.0 cm</x:v>
+        <x:v>Hydroponic Propagation Plug 4.5 cm</x:v>
       </x:c>
       <x:c r="D30" s="37" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>水培育苗块 / Hydroponic Plug</x:v>
       </x:c>
       <x:c r="E30" s="37" t="str">
-        <x:v>Top Ø 3.2 cm / Bottom Ø 2.5 cm / Height 4.0 cm</x:v>
+        <x:v>Top Ø 3.5 cm / Bottom Ø 2.2 cm / Height 4.5 cm</x:v>
       </x:c>
       <x:c r="F30" s="37" t="str">
-        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
+        <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
       </x:c>
       <x:c r="G30" s="37" t="str">
-        <x:v>Cuttings propagation and tray-fit projects requiring a 3.2 cm top diameter</x:v>
+        <x:v>Hydroponic propagation and controlled-environment nursery production</x:v>
       </x:c>
       <x:c r="H30" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1393,134 +1387,102 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J30" s="37" t="str">
-        <x:v>assets/products/CF-3240-dimensions.webp</x:v>
+        <x:v>assets/products/CF-3545-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="46" customHeight="1">
       <x:c r="A31" s="34" t="str">
-        <x:v>CF-3545</x:v>
+        <x:v>CF-3550</x:v>
       </x:c>
       <x:c r="B31" s="17" t="str">
-        <x:v>水培育苗块 4.5 cm</x:v>
+        <x:v>高型育苗块 5.3 cm</x:v>
       </x:c>
       <x:c r="C31" s="17" t="str">
-        <x:v>Hydroponic Propagation Plug 4.5 cm</x:v>
+        <x:v>Tall Nursery Plug 5.3 cm</x:v>
       </x:c>
       <x:c r="D31" s="17" t="str">
-        <x:v>水培育苗块 / Hydroponic Plug</x:v>
+        <x:v>育苗基质块 / Seedling Plug</x:v>
       </x:c>
       <x:c r="E31" s="17" t="str">
-        <x:v>Top Ø 3.5 cm / Bottom Ø 2.2 cm / Height 4.5 cm</x:v>
+        <x:v>Top Ø 3.7 cm / Bottom Ø 2.2 cm / Height 5.3 cm</x:v>
       </x:c>
       <x:c r="F31" s="17" t="str">
-        <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
+        <x:v>Deeper nursery and propagation trays with approximately 3.7 cm openings</x:v>
       </x:c>
       <x:c r="G31" s="17" t="str">
-        <x:v>Hydroponic propagation and controlled-environment nursery production</x:v>
+        <x:v>Seedlings and cuttings requiring a taller propagation format</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I31" s="17" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J31" s="17" t="str">
-        <x:v>assets/products/CF-3545-factory.webp</x:v>
+        <x:v>assets/products/CF-3550.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="46" customHeight="1">
       <x:c r="A32" s="36" t="str">
-        <x:v>CF-3550</x:v>
+        <x:v>CF-5050</x:v>
       </x:c>
       <x:c r="B32" s="37" t="str">
-        <x:v>高型育苗块 5.3 cm</x:v>
+        <x:v>50 穴扦插育苗块 5.0 cm</x:v>
       </x:c>
       <x:c r="C32" s="37" t="str">
-        <x:v>Tall Nursery Plug 5.3 cm</x:v>
+        <x:v>50-Cell Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="D32" s="37" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E32" s="37" t="str">
-        <x:v>Top Ø 3.7 cm / Bottom Ø 2.2 cm / Height 5.3 cm</x:v>
+        <x:v>Top Ø 5.0 cm / Bottom Ø 3.8 cm / Height 5.0 cm</x:v>
       </x:c>
       <x:c r="F32" s="37" t="str">
-        <x:v>Deeper nursery and propagation trays with approximately 3.7 cm openings</x:v>
+        <x:v>50-cell propagation tray</x:v>
       </x:c>
       <x:c r="G32" s="37" t="str">
-        <x:v>Seedlings and cuttings requiring a taller propagation format</x:v>
+        <x:v>Larger cuttings and commercial 50-cell nursery workflows</x:v>
       </x:c>
       <x:c r="H32" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I32" s="37" t="str">
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+      </x:c>
+      <x:c r="J32" s="37" t="str">
+        <x:v>assets/products/CF-5050-factory.webp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="46" customHeight="1">
+      <x:c r="A33" s="35" t="str">
+        <x:v>CF-7050</x:v>
+      </x:c>
+      <x:c r="B33" s="18" t="str">
+        <x:v>高型育苗块 6.8 cm</x:v>
+      </x:c>
+      <x:c r="C33" s="18" t="str">
+        <x:v>Tall Nursery Plug 6.8 cm</x:v>
+      </x:c>
+      <x:c r="D33" s="18" t="str">
+        <x:v>育苗基质块 / Seedling Plug</x:v>
+      </x:c>
+      <x:c r="E33" s="18" t="str">
+        <x:v>Top Ø 4.8 cm / Bottom Ø 3.5 cm / Height 6.8 cm</x:v>
+      </x:c>
+      <x:c r="F33" s="18" t="str">
+        <x:v>Deep nursery trays, pots or holders with approximately 4.8 cm openings</x:v>
+      </x:c>
+      <x:c r="G33" s="18" t="str">
+        <x:v>Larger seedlings, deeper rooting stages and transplant programs</x:v>
+      </x:c>
+      <x:c r="H33" s="18" t="str">
+        <x:v>Confirm after carton size and packaging format are approved.</x:v>
+      </x:c>
+      <x:c r="I33" s="18" t="str">
         <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
-      <x:c r="J32" s="37" t="str">
-        <x:v>assets/products/CF-3550.webp</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="46" customHeight="1">
-      <x:c r="A33" s="34" t="str">
-        <x:v>CF-5050</x:v>
-      </x:c>
-      <x:c r="B33" s="17" t="str">
-        <x:v>50 穴扦插育苗块 5.0 cm</x:v>
-      </x:c>
-      <x:c r="C33" s="17" t="str">
-        <x:v>50-Cell Cuttings Propagation Plug</x:v>
-      </x:c>
-      <x:c r="D33" s="17" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
-      </x:c>
-      <x:c r="E33" s="17" t="str">
-        <x:v>Top Ø 5.0 cm / Bottom Ø 3.8 cm / Height 5.0 cm</x:v>
-      </x:c>
-      <x:c r="F33" s="17" t="str">
-        <x:v>50-cell propagation tray</x:v>
-      </x:c>
-      <x:c r="G33" s="17" t="str">
-        <x:v>Larger cuttings and commercial 50-cell nursery workflows</x:v>
-      </x:c>
-      <x:c r="H33" s="17" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
-      </x:c>
-      <x:c r="I33" s="17" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
-      </x:c>
-      <x:c r="J33" s="17" t="str">
-        <x:v>assets/products/CF-5050-factory.webp</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="46" customHeight="1">
-      <x:c r="A34" s="38" t="str">
-        <x:v>CF-7050</x:v>
-      </x:c>
-      <x:c r="B34" s="39" t="str">
-        <x:v>高型育苗块 6.8 cm</x:v>
-      </x:c>
-      <x:c r="C34" s="39" t="str">
-        <x:v>Tall Nursery Plug 6.8 cm</x:v>
-      </x:c>
-      <x:c r="D34" s="39" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
-      </x:c>
-      <x:c r="E34" s="39" t="str">
-        <x:v>Top Ø 4.8 cm / Bottom Ø 3.5 cm / Height 6.8 cm</x:v>
-      </x:c>
-      <x:c r="F34" s="39" t="str">
-        <x:v>Deep nursery trays, pots or holders with approximately 4.8 cm openings</x:v>
-      </x:c>
-      <x:c r="G34" s="39" t="str">
-        <x:v>Larger seedlings, deeper rooting stages and transplant programs</x:v>
-      </x:c>
-      <x:c r="H34" s="39" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
-      </x:c>
-      <x:c r="I34" s="39" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
-      </x:c>
-      <x:c r="J34" s="39" t="str">
+      <x:c r="J33" s="18" t="str">
         <x:v>assets/products/CF-7050.webp</x:v>
       </x:c>
     </x:row>
@@ -1531,7 +1493,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3decfa7730504456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98ccd90b0b0c4737"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1545,60 +1507,60 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="40" t="str">
+      <x:c r="A1" s="38" t="str">
         <x:v>CF Series Buyer Notes | 采购说明</x:v>
       </x:c>
-      <x:c r="B1" s="40"/>
-      <x:c r="C1" s="40"/>
-      <x:c r="D1" s="40"/>
-      <x:c r="E1" s="40"/>
-      <x:c r="F1" s="40"/>
+      <x:c r="B1" s="38"/>
+      <x:c r="C1" s="38"/>
+      <x:c r="D1" s="38"/>
+      <x:c r="E1" s="38"/>
+      <x:c r="F1" s="38"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="45" t="str">
+      <x:c r="A3" s="43" t="str">
         <x:v>项目 / Item</x:v>
       </x:c>
-      <x:c r="B3" s="45" t="str">
+      <x:c r="B3" s="43" t="str">
         <x:v>说明 / Note</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
-      <x:c r="A4" s="46" t="str">
+      <x:c r="A4" s="44" t="str">
         <x:v>产品范围</x:v>
       </x:c>
-      <x:c r="B4" s="43" t="str">
-        <x:v>30 个公开 CF 型号；不含工厂内部型号映射。</x:v>
+      <x:c r="B4" s="41" t="str">
+        <x:v>29 个公开 CF 型号；不含工厂内部型号映射。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="46" t="str">
+      <x:c r="A5" s="44" t="str">
         <x:v>材料</x:v>
       </x:c>
-      <x:c r="B5" s="43" t="str">
+      <x:c r="B5" s="41" t="str">
         <x:v>Molded coconut coir and peat substrate with adjustable plant-fiber binder ratio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
-      <x:c r="A6" s="46" t="str">
+      <x:c r="A6" s="44" t="str">
         <x:v>尺寸确认</x:v>
       </x:c>
-      <x:c r="B6" s="43" t="str">
+      <x:c r="B6" s="41" t="str">
         <x:v>穴盘品牌、穴数、顶部/底部孔径和深度应在打样前按图纸或实物确认。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
-      <x:c r="A7" s="46" t="str">
+      <x:c r="A7" s="44" t="str">
         <x:v>包装与 MOQ</x:v>
       </x:c>
-      <x:c r="B7" s="43" t="str">
+      <x:c r="B7" s="41" t="str">
         <x:v>装箱数量为参考值；最终数量和 MOQ 按纸箱、零售包装、标签及运输方式确认。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="46" t="str">
+      <x:c r="A8" s="44" t="str">
         <x:v>文件支持</x:v>
       </x:c>
-      <x:c r="B8" s="43" t="str">
+      <x:c r="B8" s="41" t="str">
         <x:v>SGS report, SDS, composition statement and export-document coordination are available by project.</x:v>
       </x:c>
     </x:row>

</xml_diff>